<commit_message>
omg wow so cool wow
</commit_message>
<xml_diff>
--- a/Resources/What's my Score in MGMT 205.xlsx
+++ b/Resources/What's my Score in MGMT 205.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Courses\PErsonal Finance\MGMT 205 - PErsonal Finance\SP24 MGMT 205\General and Admin\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f4dc847ec8b5479/Documents/CWRU/Spring 2025/MGMT205/Resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F599BB49-9AC8-41B3-940F-43A09F3D2606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{F599BB49-9AC8-41B3-940F-43A09F3D2606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9597160-F259-4273-BAD1-7198348B992E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{EC70741E-6E1E-4DCA-AD69-26201168C414}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="19200" windowHeight="11170" xr2:uid="{EC70741E-6E1E-4DCA-AD69-26201168C414}"/>
   </bookViews>
   <sheets>
     <sheet name="SP24" sheetId="1" r:id="rId1"/>
@@ -529,14 +529,14 @@
         <v>3</v>
       </c>
       <c r="D5" s="2">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="F5" s="5">
         <v>0.3</v>
       </c>
       <c r="H5">
         <f>D5*F5</f>
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -708,7 +708,7 @@
       </c>
       <c r="H28" s="6">
         <f>SUM(H5:H27)</f>
-        <v>92.5</v>
+        <v>95.5</v>
       </c>
       <c r="I28" t="s">
         <v>9</v>

</xml_diff>